<commit_message>
devisthan sinchai and gh continue
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/तिनघरे बाटो स्तरोन्नति/valuation तिनघरे बाटो स्तरोन्नति.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/तिनघरे बाटो स्तरोन्नति/valuation तिनघरे बाटो स्तरोन्नति.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
     <sheet name="valuation" sheetId="14" r:id="rId2"/>
     <sheet name="WCR" sheetId="15" r:id="rId3"/>
-    <sheet name="measure" sheetId="16" r:id="rId4"/>
+    <sheet name="m" sheetId="17" r:id="rId4"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId5"/>
@@ -19,7 +19,6 @@
     <externalReference r:id="rId8"/>
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
-    <externalReference r:id="rId11"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
@@ -37,33 +36,33 @@
     <definedName name="description_310" localSheetId="0">#REF!</definedName>
     <definedName name="description_310" localSheetId="3">#REF!</definedName>
     <definedName name="description_310" localSheetId="1">#REF!</definedName>
-    <definedName name="description_310" localSheetId="2">[5]Abstract!$B$60</definedName>
+    <definedName name="description_310" localSheetId="2">[4]Abstract!$B$60</definedName>
     <definedName name="description_310">#REF!</definedName>
     <definedName name="description_312" localSheetId="0">#REF!</definedName>
     <definedName name="description_312" localSheetId="3">#REF!</definedName>
     <definedName name="description_312" localSheetId="1">#REF!</definedName>
-    <definedName name="description_312" localSheetId="2">[6]Abstract!$B$61</definedName>
+    <definedName name="description_312" localSheetId="2">[5]Abstract!$B$61</definedName>
     <definedName name="description_312">#REF!</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
     <definedName name="description_6" localSheetId="0">#REF!</definedName>
     <definedName name="description_6" localSheetId="3">#REF!</definedName>
     <definedName name="description_6" localSheetId="1">#REF!</definedName>
-    <definedName name="description_6" localSheetId="2">[5]Abstract!$B$172</definedName>
+    <definedName name="description_6" localSheetId="2">[4]Abstract!$B$172</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
     <definedName name="description_781" localSheetId="0">#REF!</definedName>
     <definedName name="description_781" localSheetId="3">#REF!</definedName>
     <definedName name="description_781" localSheetId="1">#REF!</definedName>
-    <definedName name="description_781" localSheetId="2">[7]Abstract!$B$299</definedName>
+    <definedName name="description_781" localSheetId="2">[6]Abstract!$B$299</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$46</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">measure!$A$1:$K$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">m!$A$1:$K$51</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">valuation!$A$1:$K$51</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">WCR!$A$1:$K$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">measure!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">m!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">valuation!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">WCR!$1:$12</definedName>
   </definedNames>
@@ -500,7 +499,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -590,24 +589,53 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -627,6 +655,48 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -636,86 +706,16 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -959,27 +959,6 @@
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
-      <sheetName val="Estimate"/>
-      <sheetName val="WCR"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>Project:- कालीमस्ट मन्दिर निर्माण</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
       <sheetName val="Datasheet"/>
       <sheetName val="Abstract"/>
       <sheetName val="Quantity_Sheet"/>
@@ -1040,7 +1019,7 @@
 </externalLink>
 </file>
 
-<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -1099,7 +1078,7 @@
 </externalLink>
 </file>
 
-<file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -1464,113 +1443,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
     </row>
     <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
     </row>
     <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
     </row>
     <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
     </row>
     <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="59"/>
     </row>
     <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
@@ -2294,11 +2273,11 @@
       <c r="B41" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="C41" s="43">
+      <c r="C41" s="56">
         <f>J39</f>
         <v>573377.51460942498</v>
       </c>
-      <c r="D41" s="44"/>
+      <c r="D41" s="57"/>
       <c r="E41" s="9">
         <v>100</v>
       </c>
@@ -2320,21 +2299,21 @@
       <c r="B42" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C42" s="47">
+      <c r="C42" s="60">
         <v>500000</v>
       </c>
-      <c r="D42" s="48"/>
+      <c r="D42" s="61"/>
       <c r="E42" s="9"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B43" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C43" s="47">
+      <c r="C43" s="60">
         <f>C42-C45-C46</f>
         <v>475000</v>
       </c>
-      <c r="D43" s="48"/>
+      <c r="D43" s="61"/>
       <c r="E43" s="9">
         <f>C43/C41*100</f>
         <v>82.842453339587607</v>
@@ -2344,11 +2323,11 @@
       <c r="B44" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C44" s="49">
+      <c r="C44" s="62">
         <f>C41-C43</f>
         <v>98377.514609424979</v>
       </c>
-      <c r="D44" s="49"/>
+      <c r="D44" s="62"/>
       <c r="E44" s="9">
         <f>100-E43</f>
         <v>17.157546660412393</v>
@@ -2358,11 +2337,11 @@
       <c r="B45" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C45" s="43">
+      <c r="C45" s="56">
         <f>C42*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D45" s="44"/>
+      <c r="D45" s="57"/>
       <c r="E45" s="9">
         <v>3</v>
       </c>
@@ -2371,17 +2350,24 @@
       <c r="B46" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C46" s="43">
+      <c r="C46" s="56">
         <f>C42*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D46" s="44"/>
+      <c r="D46" s="57"/>
       <c r="E46" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="A7:F7"/>
@@ -2390,13 +2376,6 @@
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="C44:D44"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2430,113 +2409,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
     </row>
     <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
     </row>
     <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
     </row>
     <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
     </row>
     <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="59"/>
     </row>
     <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
@@ -2595,7 +2574,7 @@
       <c r="B10" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="83">
         <v>1</v>
       </c>
       <c r="D10" s="33">
@@ -2604,14 +2583,14 @@
       </c>
       <c r="E10" s="33">
         <f>E22</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F10" s="33">
         <v>3</v>
       </c>
       <c r="G10" s="33">
         <f>PRODUCT(C10:F10)</f>
-        <v>46.215000000000003</v>
+        <v>45.03</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -2636,7 +2615,7 @@
       <c r="B11" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="83">
         <v>1</v>
       </c>
       <c r="D11" s="33">
@@ -2683,7 +2662,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="6">
         <f>SUM(G10:G11)</f>
-        <v>65.115000000000009</v>
+        <v>63.93</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>17</v>
@@ -2693,7 +2672,7 @@
       </c>
       <c r="J12" s="18">
         <f>G12*I12</f>
-        <v>4098.9892500000005</v>
+        <v>4024.3935000000001</v>
       </c>
       <c r="K12" s="5"/>
     </row>
@@ -2711,7 +2690,7 @@
       <c r="I13" s="17"/>
       <c r="J13" s="18">
         <f>0.13*G12*(18612)/360</f>
-        <v>437.63791500000008</v>
+        <v>429.67353000000003</v>
       </c>
       <c r="K13" s="17"/>
     </row>
@@ -2760,14 +2739,14 @@
       </c>
       <c r="E16" s="33">
         <f>E22</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F16" s="33">
         <v>0.15</v>
       </c>
       <c r="G16" s="33">
         <f>PRODUCT(C16:F16)</f>
-        <v>2.3107500000000001</v>
+        <v>2.2515000000000001</v>
       </c>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -2840,7 +2819,7 @@
       <c r="F18" s="5"/>
       <c r="G18" s="6">
         <f>SUM(G16:G17)</f>
-        <v>3.2557499999999999</v>
+        <v>3.1964999999999999</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>17</v>
@@ -2850,7 +2829,7 @@
       </c>
       <c r="J18" s="18">
         <f>G18*I18</f>
-        <v>14515.826490000001</v>
+        <v>14251.659180000001</v>
       </c>
       <c r="K18" s="5"/>
     </row>
@@ -2868,7 +2847,7 @@
       <c r="I19" s="17"/>
       <c r="J19" s="18">
         <f>0.13*G18*(14817.6)/5</f>
-        <v>1254.3024312</v>
+        <v>1231.4759184</v>
       </c>
       <c r="K19" s="17"/>
     </row>
@@ -2916,15 +2895,14 @@
         <v>7.9</v>
       </c>
       <c r="E22" s="33">
-        <f>F34/2</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F22" s="33">
         <v>0.05</v>
       </c>
       <c r="G22" s="33">
         <f>PRODUCT(C22:F22)</f>
-        <v>0.7702500000000001</v>
+        <v>0.75050000000000006</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="17"/>
@@ -3055,7 +3033,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="6">
         <f>SUM(G22:G25)</f>
-        <v>1.3615000000000002</v>
+        <v>1.3417500000000002</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>17</v>
@@ -3065,7 +3043,7 @@
       </c>
       <c r="J26" s="18">
         <f>G26*I26</f>
-        <v>14928.112290000001</v>
+        <v>14711.564205000001</v>
       </c>
       <c r="K26" s="5"/>
     </row>
@@ -3083,7 +3061,7 @@
       <c r="I27" s="17"/>
       <c r="J27" s="18">
         <f>0.13*G26*(53818.03)/15</f>
-        <v>635.03481465666675</v>
+        <v>625.82296185500013</v>
       </c>
       <c r="K27" s="17"/>
     </row>
@@ -3101,7 +3079,7 @@
       <c r="I28" s="17"/>
       <c r="J28" s="18">
         <f>0.13*G26*(21432.6)/15</f>
-        <v>252.89753579999999</v>
+        <v>249.22898910000004</v>
       </c>
       <c r="K28" s="17"/>
     </row>
@@ -3119,7 +3097,7 @@
       <c r="I29" s="17"/>
       <c r="J29" s="18">
         <f>0.13*G26*(25719.12+13573.98+4286.52)/15</f>
-        <v>514.22498945999996</v>
+        <v>506.76561117000006</v>
       </c>
       <c r="K29" s="17"/>
     </row>
@@ -3137,7 +3115,7 @@
       <c r="I30" s="17"/>
       <c r="J30" s="18">
         <f>0.13*G26*(6325.7)/15</f>
-        <v>74.641151433333334</v>
+        <v>73.558402450000003</v>
       </c>
       <c r="K30" s="17"/>
     </row>
@@ -3155,7 +3133,7 @@
       <c r="I31" s="17"/>
       <c r="J31" s="18">
         <f>0.13*G26*(310)/5</f>
-        <v>10.973690000000001</v>
+        <v>10.814505000000002</v>
       </c>
       <c r="K31" s="17"/>
     </row>
@@ -3203,15 +3181,15 @@
         <v>7.9</v>
       </c>
       <c r="E34" s="33">
-        <f>((F34/2)+0.5)/2</f>
-        <v>1.2250000000000001</v>
+        <f>(1.9+0.5)/2</f>
+        <v>1.2</v>
       </c>
       <c r="F34" s="33">
         <v>3.9</v>
       </c>
       <c r="G34" s="33">
         <f>PRODUCT(C34:F34)</f>
-        <v>37.742250000000006</v>
+        <v>36.972000000000001</v>
       </c>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
@@ -3283,7 +3261,7 @@
       <c r="F36" s="5"/>
       <c r="G36" s="6">
         <f>SUM(G34:G35)</f>
-        <v>53.492250000000006</v>
+        <v>52.722000000000001</v>
       </c>
       <c r="H36" s="7" t="s">
         <v>17</v>
@@ -3293,7 +3271,7 @@
       </c>
       <c r="J36" s="18">
         <f>G36*I36</f>
-        <v>480779.24931750004</v>
+        <v>473856.37326000002</v>
       </c>
       <c r="K36" s="5"/>
     </row>
@@ -3311,7 +3289,7 @@
       <c r="I37" s="17"/>
       <c r="J37" s="18">
         <f>0.13*G36*(5863.95)/5</f>
-        <v>8155.5728640750003</v>
+        <v>8038.1384693999989</v>
       </c>
       <c r="K37" s="17"/>
     </row>
@@ -3329,7 +3307,7 @@
       <c r="I38" s="17"/>
       <c r="J38" s="18">
         <f>0.13*G36*(6604.416)/5</f>
-        <v>9185.4118661760021</v>
+        <v>9053.1485291520003</v>
       </c>
       <c r="K38" s="17"/>
     </row>
@@ -3347,7 +3325,7 @@
       <c r="I39" s="17"/>
       <c r="J39" s="18">
         <f>0.13*G36*(14808.78)/5</f>
-        <v>20596.029010830003</v>
+        <v>20299.460978160001</v>
       </c>
       <c r="K39" s="17"/>
     </row>
@@ -3365,7 +3343,7 @@
       <c r="I40" s="17"/>
       <c r="J40" s="18">
         <f>0.13*G36*(310)/5</f>
-        <v>431.14753500000006</v>
+        <v>424.93932000000007</v>
       </c>
       <c r="K40" s="17"/>
     </row>
@@ -3438,7 +3416,7 @@
       <c r="I44" s="18"/>
       <c r="J44" s="18">
         <f>SUM(J9:J42)</f>
-        <v>556370.05115113105</v>
+        <v>548287.01735968702</v>
       </c>
       <c r="K44" s="25"/>
     </row>
@@ -3456,11 +3434,11 @@
       <c r="B46" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C46" s="43">
+      <c r="C46" s="56">
         <f>J44</f>
-        <v>556370.05115113105</v>
-      </c>
-      <c r="D46" s="44"/>
+        <v>548287.01735968702</v>
+      </c>
+      <c r="D46" s="57"/>
       <c r="E46" s="9">
         <v>100</v>
       </c>
@@ -3482,21 +3460,21 @@
       <c r="B47" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="47">
+      <c r="C47" s="60">
         <v>500000</v>
       </c>
-      <c r="D47" s="48"/>
+      <c r="D47" s="61"/>
       <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B48" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C48" s="47">
+      <c r="C48" s="60">
         <f>82.84%*C46</f>
-        <v>460896.95037359698</v>
-      </c>
-      <c r="D48" s="48"/>
+        <v>454200.96518076473</v>
+      </c>
+      <c r="D48" s="61"/>
       <c r="E48" s="9">
         <f>C48/C46*100</f>
         <v>82.84</v>
@@ -3506,11 +3484,11 @@
       <c r="B49" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="49">
+      <c r="C49" s="62">
         <f>C46-C48</f>
-        <v>95473.100777534069</v>
-      </c>
-      <c r="D49" s="49"/>
+        <v>94086.052178922284</v>
+      </c>
+      <c r="D49" s="62"/>
       <c r="E49" s="9">
         <f>100-E48</f>
         <v>17.159999999999997</v>
@@ -3520,11 +3498,11 @@
       <c r="B50" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C50" s="43">
+      <c r="C50" s="56">
         <f>C47*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D50" s="44"/>
+      <c r="D50" s="57"/>
       <c r="E50" s="9">
         <v>3</v>
       </c>
@@ -3533,17 +3511,24 @@
       <c r="B51" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C51" s="43">
+      <c r="C51" s="56">
         <f>C47*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D51" s="44"/>
+      <c r="D51" s="57"/>
       <c r="E51" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C50:D50"/>
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="A7:F7"/>
@@ -3552,13 +3537,6 @@
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -3591,775 +3569,788 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
     </row>
     <row r="2" spans="1:11" ht="24.6" x14ac:dyDescent="0.4">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="78" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-    </row>
-    <row r="3" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="52" t="s">
+      <c r="B2" s="78"/>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+    </row>
+    <row r="3" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
-      <c r="J3" s="52"/>
-      <c r="K3" s="52"/>
-    </row>
-    <row r="4" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
+      <c r="B3" s="79"/>
+      <c r="C3" s="79"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="79"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="79"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="79"/>
+    </row>
+    <row r="4" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="52"/>
+      <c r="B4" s="79"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="79"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
+      <c r="G4" s="79"/>
+      <c r="H4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
     </row>
     <row r="5" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="80" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
+      <c r="B5" s="80"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="80"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
     </row>
     <row r="6" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="55" t="s">
+      <c r="A6" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="55"/>
-      <c r="C6" s="56">
+      <c r="B6" s="38"/>
+      <c r="C6" s="81">
         <f>F34</f>
         <v>573362.97638442495</v>
       </c>
-      <c r="D6" s="57"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55" t="s">
+      <c r="D6" s="82"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="55"/>
-      <c r="J6" s="56">
+      <c r="I6" s="38"/>
+      <c r="J6" s="81">
         <f>I34</f>
-        <v>556359.07746113103</v>
-      </c>
-      <c r="K6" s="57"/>
+        <v>548276.20285468712</v>
+      </c>
+      <c r="K6" s="82"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="59"/>
-      <c r="D7" s="59"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="I7" s="61" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="F7" s="72"/>
+      <c r="G7" s="72"/>
+      <c r="I7" s="73" t="s">
         <v>49</v>
       </c>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
+      <c r="J7" s="73"/>
+      <c r="K7" s="73"/>
     </row>
     <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="62" t="str">
+      <c r="A8" s="74" t="str">
         <f>estimate!A6</f>
         <v>Project:-तिनघरे बाटो स्तरोन्नति</v>
       </c>
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="I8" s="63" t="s">
+      <c r="B8" s="74"/>
+      <c r="C8" s="74"/>
+      <c r="D8" s="74"/>
+      <c r="E8" s="74"/>
+      <c r="F8" s="74"/>
+      <c r="I8" s="75" t="s">
         <v>58</v>
       </c>
-      <c r="J8" s="63"/>
-      <c r="K8" s="63"/>
+      <c r="J8" s="75"/>
+      <c r="K8" s="75"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="64" t="str">
+      <c r="A9" s="76" t="str">
         <f>estimate!A7</f>
         <v>Location:- Shankharapur Municipality 1</v>
       </c>
-      <c r="B9" s="64"/>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
-      <c r="E9" s="64"/>
-      <c r="F9" s="64"/>
-      <c r="I9" s="63" t="s">
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="I9" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="J9" s="63"/>
-      <c r="K9" s="63"/>
+      <c r="J9" s="75"/>
+      <c r="K9" s="75"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="65" t="s">
+      <c r="B11" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="65" t="s">
+      <c r="C11" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="66" t="s">
+      <c r="D11" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="66"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66" t="s">
+      <c r="E11" s="71"/>
+      <c r="F11" s="71"/>
+      <c r="G11" s="71" t="s">
         <v>53</v>
       </c>
-      <c r="H11" s="66"/>
-      <c r="I11" s="66"/>
-      <c r="J11" s="65" t="s">
+      <c r="H11" s="71"/>
+      <c r="I11" s="71"/>
+      <c r="J11" s="70" t="s">
         <v>54</v>
       </c>
-      <c r="K11" s="67" t="s">
+      <c r="K11" s="69" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="65"/>
-      <c r="B12" s="65"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="68" t="s">
+      <c r="A12" s="70"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="68" t="s">
+      <c r="E12" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="68" t="s">
+      <c r="F12" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="68" t="s">
+      <c r="G12" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="H12" s="68" t="s">
+      <c r="H12" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="I12" s="68" t="s">
+      <c r="I12" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="65"/>
-      <c r="K12" s="67"/>
-    </row>
-    <row r="13" spans="1:11" s="53" customFormat="1" ht="140.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="69">
+      <c r="J12" s="70"/>
+      <c r="K12" s="69"/>
+    </row>
+    <row r="13" spans="1:11" s="37" customFormat="1" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="42">
         <f>estimate!A9</f>
         <v>1</v>
       </c>
-      <c r="B13" s="70" t="str">
+      <c r="B13" s="43" t="str">
         <f>estimate!B9</f>
         <v>Earthwork Excavation in Cutting., Roadway Excavation in all types of Soil by Mechanical  Means ., Road way Excavation in  all types of soil as per Drawing and technical specifications  including  removal of stumps and other deleterious matter and backfilling, all lifts and lead as per Drawing and instruction of the Engineer.</v>
       </c>
-      <c r="C13" s="71" t="str">
+      <c r="C13" s="44" t="str">
         <f>estimate!H11</f>
         <v>m3</v>
       </c>
-      <c r="D13" s="71">
+      <c r="D13" s="44">
         <f>estimate!G11</f>
         <v>83.25</v>
       </c>
-      <c r="E13" s="71">
+      <c r="E13" s="44">
         <f>estimate!I11</f>
         <v>62.95</v>
       </c>
-      <c r="F13" s="71">
+      <c r="F13" s="44">
         <f>D13*E13</f>
         <v>5240.5875000000005</v>
       </c>
-      <c r="G13" s="71">
+      <c r="G13" s="44">
         <f>valuation!G12</f>
-        <v>65.115000000000009</v>
-      </c>
-      <c r="H13" s="71">
+        <v>63.93</v>
+      </c>
+      <c r="H13" s="44">
         <f>valuation!I12</f>
         <v>62.95</v>
       </c>
-      <c r="I13" s="71">
+      <c r="I13" s="44">
         <f>G13*H13</f>
-        <v>4098.9892500000005</v>
-      </c>
-      <c r="J13" s="72">
+        <v>4024.3935000000001</v>
+      </c>
+      <c r="J13" s="45">
         <f>I13-F13</f>
-        <v>-1141.59825</v>
-      </c>
-      <c r="K13" s="73"/>
-    </row>
-    <row r="14" spans="1:11" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="69"/>
-      <c r="B14" s="74" t="str">
+        <v>-1216.1940000000004</v>
+      </c>
+      <c r="K13" s="46"/>
+    </row>
+    <row r="14" spans="1:11" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="42"/>
+      <c r="B14" s="47" t="str">
         <f>estimate!B12</f>
         <v>-13% VAT for materials</v>
       </c>
-      <c r="C14" s="71"/>
-      <c r="D14" s="71"/>
-      <c r="E14" s="71"/>
-      <c r="F14" s="71">
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44">
         <f>estimate!J12</f>
         <v>559.52324999999996</v>
       </c>
-      <c r="G14" s="71"/>
-      <c r="H14" s="71"/>
-      <c r="I14" s="71">
+      <c r="G14" s="44"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44">
         <f>valuation!J13</f>
-        <v>437.63791500000008</v>
-      </c>
-      <c r="J14" s="72">
+        <v>429.67353000000003</v>
+      </c>
+      <c r="J14" s="45">
         <f>I14-F14</f>
-        <v>-121.88533499999988</v>
-      </c>
-      <c r="K14" s="73"/>
-    </row>
-    <row r="15" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="75"/>
-      <c r="B15" s="76"/>
-      <c r="C15" s="71"/>
-      <c r="D15" s="71"/>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="71"/>
-      <c r="I15" s="71"/>
-      <c r="J15" s="72"/>
-      <c r="K15" s="73"/>
-    </row>
-    <row r="16" spans="1:11" s="53" customFormat="1" ht="78" x14ac:dyDescent="0.3">
-      <c r="A16" s="69">
+        <v>-129.84971999999993</v>
+      </c>
+      <c r="K14" s="46"/>
+    </row>
+    <row r="15" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="48"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="45"/>
+      <c r="K15" s="46"/>
+    </row>
+    <row r="16" spans="1:11" s="37" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A16" s="42">
         <f>estimate!A14</f>
         <v>2</v>
       </c>
-      <c r="B16" s="70" t="str">
+      <c r="B16" s="43" t="str">
         <f>estimate!B14</f>
         <v>Providing and laying of hand pack locally available Stone soling with 150 to 200 mm thick stones and packing with smaller stone on prepared surface as per Drawing and Technical Specifications.</v>
       </c>
-      <c r="C16" s="71" t="str">
+      <c r="C16" s="44" t="str">
         <f>estimate!H16</f>
         <v>m3</v>
       </c>
-      <c r="D16" s="71">
+      <c r="D16" s="44">
         <f>estimate!G16</f>
         <v>4.1624999999999996</v>
       </c>
-      <c r="E16" s="71">
+      <c r="E16" s="44">
         <f>estimate!I16</f>
         <v>4458.5200000000004</v>
       </c>
-      <c r="F16" s="71">
+      <c r="F16" s="44">
         <f>D16*E16</f>
         <v>18558.589500000002</v>
       </c>
-      <c r="G16" s="71">
+      <c r="G16" s="44">
         <f>valuation!G18</f>
-        <v>3.2557499999999999</v>
-      </c>
-      <c r="H16" s="71">
+        <v>3.1964999999999999</v>
+      </c>
+      <c r="H16" s="44">
         <f>valuation!I18</f>
         <v>4458.5200000000004</v>
       </c>
-      <c r="I16" s="71">
+      <c r="I16" s="44">
         <f>G16*H16</f>
-        <v>14515.826490000001</v>
-      </c>
-      <c r="J16" s="72">
+        <v>14251.659180000001</v>
+      </c>
+      <c r="J16" s="45">
         <f>I16-F16</f>
-        <v>-4042.7630100000006</v>
-      </c>
-      <c r="K16" s="73"/>
-    </row>
-    <row r="17" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="69"/>
-      <c r="B17" s="74" t="str">
+        <v>-4306.9303200000013</v>
+      </c>
+      <c r="K16" s="46"/>
+    </row>
+    <row r="17" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="42"/>
+      <c r="B17" s="47" t="str">
         <f>estimate!B17</f>
         <v>-13% VAT for materials</v>
       </c>
-      <c r="C17" s="71"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71">
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44">
         <f>estimate!J17</f>
         <v>1603.6347599999999</v>
       </c>
-      <c r="G17" s="71"/>
-      <c r="H17" s="71"/>
-      <c r="I17" s="71">
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="44">
         <f>valuation!J19</f>
-        <v>1254.3024312</v>
-      </c>
-      <c r="J17" s="72">
+        <v>1231.4759184</v>
+      </c>
+      <c r="J17" s="45">
         <f>I17-F17</f>
-        <v>-349.33232879999991</v>
-      </c>
-      <c r="K17" s="73"/>
-    </row>
-    <row r="18" spans="1:13" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="75"/>
-      <c r="B18" s="76"/>
-      <c r="C18" s="71"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="71"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="71"/>
-      <c r="H18" s="71"/>
-      <c r="I18" s="71"/>
-      <c r="J18" s="72"/>
-      <c r="K18" s="73"/>
-    </row>
-    <row r="19" spans="1:13" s="53" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="69">
+        <v>-372.15884159999996</v>
+      </c>
+      <c r="K17" s="46"/>
+    </row>
+    <row r="18" spans="1:13" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="48"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="46"/>
+    </row>
+    <row r="19" spans="1:13" s="37" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="42">
         <f>estimate!A19</f>
         <v>3</v>
       </c>
-      <c r="B19" s="70" t="str">
+      <c r="B19" s="43" t="str">
         <f>estimate!B19</f>
         <v>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications, PCC Grade M 15</v>
       </c>
-      <c r="C19" s="71" t="str">
+      <c r="C19" s="44" t="str">
         <f>estimate!H22</f>
         <v>m3</v>
       </c>
-      <c r="D19" s="71">
+      <c r="D19" s="44">
         <f>estimate!G22</f>
         <v>1.8037500000000002</v>
       </c>
-      <c r="E19" s="71">
+      <c r="E19" s="44">
         <f>estimate!I22</f>
         <v>10964.46</v>
       </c>
-      <c r="F19" s="71">
+      <c r="F19" s="44">
         <f>D19*E19</f>
         <v>19777.144725000002</v>
       </c>
-      <c r="G19" s="71">
+      <c r="G19" s="44">
         <f>valuation!G26</f>
-        <v>1.3615000000000002</v>
-      </c>
-      <c r="H19" s="71">
+        <v>1.3417500000000002</v>
+      </c>
+      <c r="H19" s="44">
         <f>valuation!I26</f>
         <v>10964.46</v>
       </c>
-      <c r="I19" s="71">
+      <c r="I19" s="44">
         <f>G19*H19</f>
-        <v>14928.112290000001</v>
-      </c>
-      <c r="J19" s="72">
+        <v>14711.564205000001</v>
+      </c>
+      <c r="J19" s="45">
         <f>I19-F19</f>
-        <v>-4849.032435000001</v>
-      </c>
-      <c r="K19" s="73"/>
-    </row>
-    <row r="20" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="69"/>
-      <c r="B20" s="74" t="str">
+        <v>-5065.5805200000013</v>
+      </c>
+      <c r="K19" s="46"/>
+    </row>
+    <row r="20" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="42"/>
+      <c r="B20" s="47" t="str">
         <f>estimate!B23</f>
         <v>-13% VAT for cement</v>
       </c>
-      <c r="C20" s="71"/>
-      <c r="D20" s="71"/>
-      <c r="E20" s="71"/>
-      <c r="F20" s="71">
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44">
         <f>estimate!J23</f>
         <v>841.31035397500023</v>
       </c>
-      <c r="G20" s="71"/>
-      <c r="H20" s="71"/>
-      <c r="I20" s="71">
+      <c r="G20" s="44"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="44">
         <f>valuation!J27</f>
-        <v>635.03481465666675</v>
-      </c>
-      <c r="J20" s="72">
+        <v>625.82296185500013</v>
+      </c>
+      <c r="J20" s="45">
         <f t="shared" ref="J20:J23" si="0">I20-F20</f>
-        <v>-206.27553931833347</v>
-      </c>
-      <c r="K20" s="73"/>
-    </row>
-    <row r="21" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="69"/>
-      <c r="B21" s="74" t="str">
+        <v>-215.4873921200001</v>
+      </c>
+      <c r="K20" s="46"/>
+    </row>
+    <row r="21" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="42"/>
+      <c r="B21" s="47" t="str">
         <f>estimate!B24</f>
         <v>-13% VAT for sand</v>
       </c>
-      <c r="C21" s="71"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71">
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44">
         <f>estimate!J24</f>
         <v>335.0451195</v>
       </c>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
-      <c r="I21" s="71">
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44">
         <f>valuation!J28</f>
-        <v>252.89753579999999</v>
-      </c>
-      <c r="J21" s="72">
+        <v>249.22898910000004</v>
+      </c>
+      <c r="J21" s="45">
         <f t="shared" si="0"/>
-        <v>-82.147583700000013</v>
-      </c>
-      <c r="K21" s="73"/>
-    </row>
-    <row r="22" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="69"/>
-      <c r="B22" s="74" t="str">
+        <v>-85.816130399999963</v>
+      </c>
+      <c r="K21" s="46"/>
+    </row>
+    <row r="22" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A22" s="42"/>
+      <c r="B22" s="47" t="str">
         <f>estimate!B25</f>
         <v>-13% VAT for aggregate</v>
       </c>
-      <c r="C22" s="71"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="71">
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44">
         <f>estimate!J25</f>
         <v>681.25840964999998</v>
       </c>
-      <c r="G22" s="71"/>
-      <c r="H22" s="71"/>
-      <c r="I22" s="71">
+      <c r="G22" s="44"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="44">
         <f>valuation!J29</f>
-        <v>514.22498945999996</v>
-      </c>
-      <c r="J22" s="72">
+        <v>506.76561117000006</v>
+      </c>
+      <c r="J22" s="45">
         <f t="shared" si="0"/>
-        <v>-167.03342019000002</v>
-      </c>
-      <c r="K22" s="73"/>
-    </row>
-    <row r="23" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="69"/>
-      <c r="B23" s="74" t="str">
+        <v>-174.49279847999992</v>
+      </c>
+      <c r="K22" s="46"/>
+    </row>
+    <row r="23" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="42"/>
+      <c r="B23" s="47" t="str">
         <f>estimate!B26</f>
         <v>-13% VAT for formworks</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="71"/>
-      <c r="F23" s="71">
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44">
         <f>estimate!J26</f>
         <v>98.886505250000013</v>
       </c>
-      <c r="G23" s="71"/>
-      <c r="H23" s="71"/>
-      <c r="I23" s="71">
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44">
         <f>valuation!J30</f>
-        <v>74.641151433333334</v>
-      </c>
-      <c r="J23" s="72">
+        <v>73.558402450000003</v>
+      </c>
+      <c r="J23" s="45">
         <f t="shared" si="0"/>
-        <v>-24.245353816666679</v>
-      </c>
-      <c r="K23" s="73"/>
-    </row>
-    <row r="24" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="69"/>
-      <c r="B24" s="74" t="str">
+        <v>-25.328102800000011</v>
+      </c>
+      <c r="K23" s="46"/>
+    </row>
+    <row r="24" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A24" s="42"/>
+      <c r="B24" s="47" t="str">
         <f>estimate!B27</f>
         <v>-13% VAT for water</v>
       </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="71"/>
-      <c r="F24" s="71"/>
-      <c r="G24" s="71"/>
-      <c r="H24" s="71"/>
-      <c r="I24" s="71"/>
-      <c r="J24" s="72"/>
-      <c r="K24" s="73"/>
-    </row>
-    <row r="25" spans="1:13" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="75"/>
-      <c r="B25" s="76"/>
-      <c r="C25" s="71"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="71"/>
-      <c r="F25" s="71"/>
-      <c r="G25" s="71"/>
-      <c r="H25" s="71"/>
-      <c r="I25" s="71"/>
-      <c r="J25" s="72"/>
-      <c r="K25" s="73"/>
-    </row>
-    <row r="26" spans="1:13" s="53" customFormat="1" ht="78" x14ac:dyDescent="0.3">
-      <c r="A26" s="69">
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="45"/>
+      <c r="K24" s="46"/>
+    </row>
+    <row r="25" spans="1:13" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="48"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="45"/>
+      <c r="K25" s="46"/>
+    </row>
+    <row r="26" spans="1:13" s="37" customFormat="1" ht="78" x14ac:dyDescent="0.3">
+      <c r="A26" s="42">
         <f>estimate!A29</f>
         <v>4</v>
       </c>
-      <c r="B26" s="70" t="str">
+      <c r="B26" s="43" t="str">
         <f>estimate!B29</f>
         <v>Random Rubble Masonry, Providing and laying of Stone Masonry Work in Cement Mortar 1:6 in Foundation complete as per Drawing and Technical Specifications., Using Concrete Mixer</v>
       </c>
-      <c r="C26" s="71" t="str">
+      <c r="C26" s="44" t="str">
         <f>estimate!H31</f>
         <v>m3</v>
       </c>
-      <c r="D26" s="71">
+      <c r="D26" s="44">
         <f>estimate!G31</f>
         <v>54.112499999999997</v>
       </c>
-      <c r="E26" s="71">
+      <c r="E26" s="44">
         <f>estimate!I31</f>
         <v>8987.83</v>
       </c>
-      <c r="F26" s="71">
+      <c r="F26" s="44">
         <f>D26*E26</f>
         <v>486353.95087499998</v>
       </c>
-      <c r="G26" s="71">
+      <c r="G26" s="44">
         <f>valuation!G36</f>
-        <v>53.492250000000006</v>
-      </c>
-      <c r="H26" s="71">
+        <v>52.722000000000001</v>
+      </c>
+      <c r="H26" s="44">
         <f>valuation!I36</f>
         <v>8987.83</v>
       </c>
-      <c r="I26" s="71">
+      <c r="I26" s="44">
         <f>G26*H26</f>
-        <v>480779.24931750004</v>
-      </c>
-      <c r="J26" s="72">
+        <v>473856.37326000002</v>
+      </c>
+      <c r="J26" s="45">
         <f>I26-F26</f>
-        <v>-5574.7015574999386</v>
-      </c>
-      <c r="K26" s="73"/>
-    </row>
-    <row r="27" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="69"/>
-      <c r="B27" s="74" t="str">
+        <v>-12497.577614999958</v>
+      </c>
+      <c r="K26" s="46"/>
+    </row>
+    <row r="27" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="42"/>
+      <c r="B27" s="47" t="str">
         <f>estimate!B32</f>
         <v>-13% VAT for cement</v>
       </c>
-      <c r="C27" s="71"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="71"/>
-      <c r="F27" s="71">
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44">
         <f>estimate!J32</f>
         <v>8250.1378537500004</v>
       </c>
-      <c r="G27" s="71"/>
-      <c r="H27" s="71"/>
-      <c r="I27" s="71">
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44">
         <f>valuation!J37</f>
-        <v>8155.5728640750003</v>
-      </c>
-      <c r="J27" s="72">
+        <v>8038.1384693999989</v>
+      </c>
+      <c r="J27" s="45">
         <f>I27-F27</f>
-        <v>-94.564989675000106</v>
-      </c>
-      <c r="K27" s="73"/>
-    </row>
-    <row r="28" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="69"/>
-      <c r="B28" s="74" t="str">
+        <v>-211.99938435000149</v>
+      </c>
+      <c r="K27" s="46"/>
+    </row>
+    <row r="28" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="42"/>
+      <c r="B28" s="47" t="str">
         <f>estimate!B33</f>
         <v>-13% VAT for sand</v>
       </c>
-      <c r="C28" s="71"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="71">
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44">
         <f>estimate!J33</f>
         <v>9291.9179808000008</v>
       </c>
-      <c r="G28" s="71"/>
-      <c r="H28" s="71"/>
-      <c r="I28" s="71">
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44">
         <f>valuation!J38</f>
-        <v>9185.4118661760021</v>
-      </c>
-      <c r="J28" s="72">
+        <v>9053.1485291520003</v>
+      </c>
+      <c r="J28" s="45">
         <f t="shared" ref="J28:J30" si="1">I28-F28</f>
-        <v>-106.50611462399866</v>
-      </c>
-      <c r="K28" s="73"/>
-    </row>
-    <row r="29" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="69"/>
-      <c r="B29" s="74" t="str">
+        <v>-238.76945164800054</v>
+      </c>
+      <c r="K28" s="46"/>
+    </row>
+    <row r="29" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="42"/>
+      <c r="B29" s="47" t="str">
         <f>estimate!B34</f>
         <v>-13% VAT for stone</v>
       </c>
-      <c r="C29" s="71"/>
-      <c r="D29" s="71"/>
-      <c r="E29" s="71"/>
-      <c r="F29" s="71">
+      <c r="C29" s="44"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44">
         <f>estimate!J34</f>
         <v>20834.842801500003</v>
       </c>
-      <c r="G29" s="71"/>
-      <c r="H29" s="71"/>
-      <c r="I29" s="71">
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="44">
         <f>valuation!J39</f>
-        <v>20596.029010830003</v>
-      </c>
-      <c r="J29" s="72">
+        <v>20299.460978160001</v>
+      </c>
+      <c r="J29" s="45">
         <f t="shared" si="1"/>
-        <v>-238.81379066999943</v>
-      </c>
-      <c r="K29" s="73"/>
-    </row>
-    <row r="30" spans="1:13" s="53" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="69"/>
-      <c r="B30" s="74" t="str">
+        <v>-535.38182334000157</v>
+      </c>
+      <c r="K29" s="46"/>
+    </row>
+    <row r="30" spans="1:13" s="37" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="42"/>
+      <c r="B30" s="47" t="str">
         <f>estimate!B35</f>
         <v>-13% VAT for water</v>
       </c>
-      <c r="C30" s="71"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="71"/>
-      <c r="F30" s="71">
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44">
         <f>estimate!J35</f>
         <v>436.14675</v>
       </c>
-      <c r="G30" s="71"/>
-      <c r="H30" s="71"/>
-      <c r="I30" s="71">
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44">
         <f>valuation!J40</f>
-        <v>431.14753500000006</v>
-      </c>
-      <c r="J30" s="72">
+        <v>424.93932000000007</v>
+      </c>
+      <c r="J30" s="45">
         <f t="shared" si="1"/>
-        <v>-4.9992149999999356</v>
-      </c>
-      <c r="K30" s="73"/>
-    </row>
-    <row r="31" spans="1:13" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="75"/>
-      <c r="B31" s="76"/>
-      <c r="C31" s="71"/>
-      <c r="D31" s="71"/>
-      <c r="E31" s="71"/>
-      <c r="F31" s="71"/>
-      <c r="G31" s="71"/>
-      <c r="H31" s="71"/>
-      <c r="I31" s="71"/>
-      <c r="J31" s="72"/>
-      <c r="K31" s="73"/>
-      <c r="M31" s="77"/>
-    </row>
-    <row r="32" spans="1:13" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="69">
+        <v>-11.207429999999931</v>
+      </c>
+      <c r="K30" s="46"/>
+    </row>
+    <row r="31" spans="1:13" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="48"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="45"/>
+      <c r="K31" s="46"/>
+      <c r="M31" s="50"/>
+    </row>
+    <row r="32" spans="1:13" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="42">
         <f>estimate!A37</f>
         <v>5</v>
       </c>
-      <c r="B32" s="78" t="str">
+      <c r="B32" s="51" t="str">
         <f>estimate!B37</f>
         <v>Information board (सुचना पाटि)</v>
       </c>
-      <c r="C32" s="71" t="str">
+      <c r="C32" s="44" t="str">
         <f>estimate!H37</f>
         <v>no.</v>
       </c>
-      <c r="D32" s="71">
+      <c r="D32" s="44">
         <f>estimate!G37</f>
         <v>1</v>
       </c>
-      <c r="E32" s="71">
+      <c r="E32" s="44">
         <f>estimate!I37</f>
         <v>500</v>
       </c>
-      <c r="F32" s="71">
+      <c r="F32" s="44">
         <f>D32*E32</f>
         <v>500</v>
       </c>
-      <c r="G32" s="71">
+      <c r="G32" s="44">
         <f>valuation!G42</f>
         <v>1</v>
       </c>
-      <c r="H32" s="71">
+      <c r="H32" s="44">
         <f>valuation!I42</f>
         <v>500</v>
       </c>
-      <c r="I32" s="71">
+      <c r="I32" s="44">
         <f>G32*H32</f>
         <v>500</v>
       </c>
-      <c r="J32" s="72">
+      <c r="J32" s="45">
         <f>I32-F32</f>
         <v>0</v>
       </c>
-      <c r="K32" s="73"/>
-    </row>
-    <row r="33" spans="1:11" s="53" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="76"/>
-      <c r="B33" s="76"/>
-      <c r="C33" s="71"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="71"/>
-      <c r="F33" s="71"/>
-      <c r="G33" s="71"/>
-      <c r="H33" s="71"/>
-      <c r="I33" s="71"/>
-      <c r="J33" s="72"/>
-      <c r="K33" s="73"/>
+      <c r="K32" s="46"/>
+    </row>
+    <row r="33" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="49"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="44"/>
+      <c r="D33" s="44"/>
+      <c r="E33" s="44"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="44"/>
+      <c r="H33" s="44"/>
+      <c r="I33" s="44"/>
+      <c r="J33" s="45"/>
+      <c r="K33" s="46"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="79"/>
-      <c r="B34" s="80" t="s">
+      <c r="A34" s="52"/>
+      <c r="B34" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="80"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81">
+      <c r="C34" s="53"/>
+      <c r="D34" s="54"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="54">
         <f>SUM(F13:F32)</f>
         <v>573362.97638442495</v>
       </c>
-      <c r="G34" s="81"/>
-      <c r="H34" s="81"/>
-      <c r="I34" s="81">
+      <c r="G34" s="54"/>
+      <c r="H34" s="54"/>
+      <c r="I34" s="54">
         <f>SUM(I13:I32)</f>
-        <v>556359.07746113103</v>
-      </c>
-      <c r="J34" s="82">
+        <v>548276.20285468712</v>
+      </c>
+      <c r="J34" s="55">
         <f>I34-F34</f>
-        <v>-17003.89892329392</v>
-      </c>
-      <c r="K34" s="79"/>
+        <v>-25086.773529737839</v>
+      </c>
+      <c r="K34" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="I9:K9"/>
     <mergeCell ref="K11:K12"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
@@ -4367,19 +4358,6 @@
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4406,121 +4384,121 @@
     <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
     <col min="7" max="7" width="9.109375" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" style="19" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="19" hidden="1" customWidth="1"/>
     <col min="11" max="12" width="9.109375" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
     <col min="17" max="16384" width="9.109375" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
     </row>
     <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="67"/>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67"/>
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
     </row>
     <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
     </row>
     <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="64"/>
+      <c r="K6" s="64"/>
     </row>
     <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="59"/>
     </row>
     <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
@@ -4579,7 +4557,7 @@
       <c r="B10" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="83">
         <v>1</v>
       </c>
       <c r="D10" s="33">
@@ -4588,14 +4566,14 @@
       </c>
       <c r="E10" s="33">
         <f>E22</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F10" s="33">
         <v>3</v>
       </c>
       <c r="G10" s="33">
         <f>PRODUCT(C10:F10)</f>
-        <v>46.215000000000003</v>
+        <v>45.03</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -4620,7 +4598,7 @@
       <c r="B11" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="83">
         <v>1</v>
       </c>
       <c r="D11" s="33">
@@ -4667,7 +4645,7 @@
       <c r="F12" s="5"/>
       <c r="G12" s="6">
         <f>SUM(G10:G11)</f>
-        <v>65.115000000000009</v>
+        <v>63.93</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>17</v>
@@ -4677,11 +4655,11 @@
       </c>
       <c r="J12" s="18">
         <f>G12*I12</f>
-        <v>4098.9892500000005</v>
+        <v>4024.3935000000001</v>
       </c>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16"/>
       <c r="B13" s="32" t="s">
         <v>23</v>
@@ -4695,7 +4673,7 @@
       <c r="I13" s="17"/>
       <c r="J13" s="18">
         <f>0.13*G12*(18612)/360</f>
-        <v>437.63791500000008</v>
+        <v>429.67353000000003</v>
       </c>
       <c r="K13" s="17"/>
     </row>
@@ -4744,14 +4722,14 @@
       </c>
       <c r="E16" s="33">
         <f>E22</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F16" s="33">
         <v>0.15</v>
       </c>
       <c r="G16" s="33">
         <f>PRODUCT(C16:F16)</f>
-        <v>2.3107500000000001</v>
+        <v>2.2515000000000001</v>
       </c>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
@@ -4824,7 +4802,7 @@
       <c r="F18" s="5"/>
       <c r="G18" s="6">
         <f>SUM(G16:G17)</f>
-        <v>3.2557499999999999</v>
+        <v>3.1964999999999999</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>17</v>
@@ -4834,11 +4812,11 @@
       </c>
       <c r="J18" s="18">
         <f>G18*I18</f>
-        <v>14515.826490000001</v>
+        <v>14251.659180000001</v>
       </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
       <c r="B19" s="32" t="s">
         <v>23</v>
@@ -4852,7 +4830,7 @@
       <c r="I19" s="17"/>
       <c r="J19" s="18">
         <f>0.13*G18*(14817.6)/5</f>
-        <v>1254.3024312</v>
+        <v>1231.4759184</v>
       </c>
       <c r="K19" s="17"/>
     </row>
@@ -4900,15 +4878,14 @@
         <v>7.9</v>
       </c>
       <c r="E22" s="33">
-        <f>F34/2</f>
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="F22" s="33">
         <v>0.05</v>
       </c>
       <c r="G22" s="33">
         <f>PRODUCT(C22:F22)</f>
-        <v>0.7702500000000001</v>
+        <v>0.75050000000000006</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22" s="17"/>
@@ -5039,7 +5016,7 @@
       <c r="F26" s="5"/>
       <c r="G26" s="6">
         <f>SUM(G22:G25)</f>
-        <v>1.3615000000000002</v>
+        <v>1.3417500000000002</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>17</v>
@@ -5049,11 +5026,11 @@
       </c>
       <c r="J26" s="18">
         <f>G26*I26</f>
-        <v>14928.112290000001</v>
+        <v>14711.564205000001</v>
       </c>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
         <v>33</v>
@@ -5067,11 +5044,11 @@
       <c r="I27" s="17"/>
       <c r="J27" s="18">
         <f>0.13*G26*(53818.03)/15</f>
-        <v>635.03481465666675</v>
+        <v>625.82296185500013</v>
       </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="16"/>
       <c r="B28" s="32" t="s">
         <v>34</v>
@@ -5085,11 +5062,11 @@
       <c r="I28" s="17"/>
       <c r="J28" s="18">
         <f>0.13*G26*(21432.6)/15</f>
-        <v>252.89753579999999</v>
+        <v>249.22898910000004</v>
       </c>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="16"/>
       <c r="B29" s="32" t="s">
         <v>35</v>
@@ -5103,11 +5080,11 @@
       <c r="I29" s="17"/>
       <c r="J29" s="18">
         <f>0.13*G26*(25719.12+13573.98+4286.52)/15</f>
-        <v>514.22498945999996</v>
+        <v>506.76561117000006</v>
       </c>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="s">
         <v>36</v>
@@ -5121,11 +5098,11 @@
       <c r="I30" s="17"/>
       <c r="J30" s="18">
         <f>0.13*G26*(6325.7)/15</f>
-        <v>74.641151433333334</v>
+        <v>73.558402450000003</v>
       </c>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="16"/>
       <c r="B31" s="32" t="s">
         <v>40</v>
@@ -5139,7 +5116,7 @@
       <c r="I31" s="17"/>
       <c r="J31" s="18">
         <f>0.13*G26*(310)/5</f>
-        <v>10.973690000000001</v>
+        <v>10.814505000000002</v>
       </c>
       <c r="K31" s="17"/>
     </row>
@@ -5187,7 +5164,7 @@
         <v>7.9</v>
       </c>
       <c r="E34" s="33">
-        <f>((F34/2)+0.45)/2</f>
+        <f>(1.9+0.5)/2</f>
         <v>1.2</v>
       </c>
       <c r="F34" s="33">
@@ -5228,15 +5205,15 @@
         <v>3.15</v>
       </c>
       <c r="E35" s="33">
-        <f>((F35/2)+0.45)/2</f>
-        <v>1.2250000000000001</v>
+        <f>((F35/2)+0.5)/2</f>
+        <v>1.25</v>
       </c>
       <c r="F35" s="33">
         <v>4</v>
       </c>
       <c r="G35" s="33">
         <f>PRODUCT(C35:F35)</f>
-        <v>15.435</v>
+        <v>15.75</v>
       </c>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
@@ -5267,7 +5244,7 @@
       <c r="F36" s="5"/>
       <c r="G36" s="6">
         <f>SUM(G34:G35)</f>
-        <v>52.407000000000004</v>
+        <v>52.722000000000001</v>
       </c>
       <c r="H36" s="7" t="s">
         <v>17</v>
@@ -5277,11 +5254,11 @@
       </c>
       <c r="J36" s="18">
         <f>G36*I36</f>
-        <v>471025.20681</v>
+        <v>473856.37326000002</v>
       </c>
       <c r="K36" s="5"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
         <v>33</v>
@@ -5295,11 +5272,11 @@
       <c r="I37" s="17"/>
       <c r="J37" s="18">
         <f>0.13*G36*(5863.95)/5</f>
-        <v>7990.1127189000008</v>
+        <v>8038.1384693999989</v>
       </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
         <v>34</v>
@@ -5313,11 +5290,11 @@
       <c r="I38" s="17"/>
       <c r="J38" s="18">
         <f>0.13*G36*(6604.416)/5</f>
-        <v>8999.0583621120004</v>
+        <v>9053.1485291520003</v>
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="16"/>
       <c r="B39" s="32" t="s">
         <v>38</v>
@@ -5331,11 +5308,11 @@
       <c r="I39" s="17"/>
       <c r="J39" s="18">
         <f>0.13*G36*(14808.78)/5</f>
-        <v>20178.177069960002</v>
+        <v>20299.460978160001</v>
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="16"/>
       <c r="B40" s="32" t="s">
         <v>40</v>
@@ -5349,7 +5326,7 @@
       <c r="I40" s="17"/>
       <c r="J40" s="18">
         <f>0.13*G36*(310)/5</f>
-        <v>422.40042000000005</v>
+        <v>424.93932000000007</v>
       </c>
       <c r="K40" s="17"/>
     </row>
@@ -5422,7 +5399,7 @@
       <c r="I44" s="18"/>
       <c r="J44" s="18">
         <f>SUM(J9:J42)</f>
-        <v>545837.59593852202</v>
+        <v>548287.01735968702</v>
       </c>
       <c r="K44" s="25"/>
     </row>
@@ -5438,13 +5415,13 @@
     <row r="46" spans="1:19" s="20" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="26"/>
       <c r="B46" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C46" s="43">
+        <v>61</v>
+      </c>
+      <c r="C46" s="56">
         <f>J44</f>
-        <v>545837.59593852202</v>
-      </c>
-      <c r="D46" s="44"/>
+        <v>548287.01735968702</v>
+      </c>
+      <c r="D46" s="57"/>
       <c r="E46" s="9">
         <v>100</v>
       </c>
@@ -5466,49 +5443,49 @@
       <c r="B47" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C47" s="47">
+      <c r="C47" s="60">
         <v>500000</v>
       </c>
-      <c r="D47" s="48"/>
+      <c r="D47" s="61"/>
       <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="B48" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C48" s="47">
-        <f>C47-C50-C51</f>
-        <v>475000</v>
-      </c>
-      <c r="D48" s="48"/>
+      <c r="C48" s="60">
+        <f>82.84%*C46</f>
+        <v>454200.96518076473</v>
+      </c>
+      <c r="D48" s="61"/>
       <c r="E48" s="9">
         <f>C48/C46*100</f>
-        <v>87.022221176113263</v>
+        <v>82.84</v>
       </c>
     </row>
     <row r="49" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B49" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="49">
+      <c r="C49" s="62">
         <f>C46-C48</f>
-        <v>70837.595938522019</v>
-      </c>
-      <c r="D49" s="49"/>
+        <v>94086.052178922284</v>
+      </c>
+      <c r="D49" s="62"/>
       <c r="E49" s="9">
         <f>100-E48</f>
-        <v>12.977778823886737</v>
+        <v>17.159999999999997</v>
       </c>
     </row>
     <row r="50" spans="2:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="B50" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C50" s="43">
+      <c r="C50" s="56">
         <f>C47*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D50" s="44"/>
+      <c r="D50" s="57"/>
       <c r="E50" s="9">
         <v>3</v>
       </c>
@@ -5517,11 +5494,11 @@
       <c r="B51" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C51" s="43">
+      <c r="C51" s="56">
         <f>C47*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D51" s="44"/>
+      <c r="D51" s="57"/>
       <c r="E51" s="9">
         <v>2</v>
       </c>
@@ -5545,12 +5522,9 @@
     <mergeCell ref="H6:K6"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
-  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="95" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="32" max="10" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>